<commit_message>
ADDED new prop to sites
</commit_message>
<xml_diff>
--- a/test/fixtures/business_example_v2.xlsx
+++ b/test/fixtures/business_example_v2.xlsx
@@ -10,14 +10,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion1">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataSignature="AMtx7mgVlRucMlGq9VKc43jj6b4l/2Ko2g=="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataSignature="AMtx7mjkLeq5sDy30Z7Dy9UQPiEyKs2yjA=="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="46">
   <si>
     <t>businessName</t>
   </si>
@@ -61,6 +61,9 @@
     <t>stateId</t>
   </si>
   <si>
+    <t>currencyCode</t>
+  </si>
+  <si>
     <t>password</t>
   </si>
   <si>
@@ -94,6 +97,9 @@
     <t>sd541</t>
   </si>
   <si>
+    <t>USD</t>
+  </si>
+  <si>
     <t>89651sasf</t>
   </si>
   <si>
@@ -116,6 +122,9 @@
   </si>
   <si>
     <t>mail23@mail.com</t>
+  </si>
+  <si>
+    <t>GBP</t>
   </si>
   <si>
     <t>4q9wf8q9</t>
@@ -186,11 +195,14 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -427,7 +439,7 @@
     <col customWidth="1" min="11" max="11" width="11.14"/>
     <col customWidth="1" min="12" max="12" width="18.29"/>
     <col customWidth="1" min="13" max="13" width="13.43"/>
-    <col customWidth="1" min="14" max="21" width="8.71"/>
+    <col customWidth="1" min="14" max="22" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -473,45 +485,48 @@
       <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="2" t="s">
         <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E2" s="2" t="s">
         <v>19</v>
       </c>
+      <c r="E2" s="3" t="s">
+        <v>20</v>
+      </c>
       <c r="F2" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H2" s="1">
         <v>1.223334444E9</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="L2" s="3">
+        <v>25</v>
+      </c>
+      <c r="L2" s="4">
         <v>43862.0</v>
       </c>
       <c r="M2" s="1">
@@ -520,45 +535,48 @@
       <c r="N2" s="1">
         <v>2.0</v>
       </c>
-      <c r="O2" s="1" t="s">
-        <v>25</v>
+      <c r="O2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>32</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H3" s="1">
         <v>1.223334444E9</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="K3" s="4">
+        <v>24</v>
+      </c>
+      <c r="K3" s="5">
         <v>5498.0</v>
       </c>
-      <c r="L3" s="3">
+      <c r="L3" s="4">
         <v>43862.0</v>
       </c>
       <c r="M3" s="1">
@@ -567,8 +585,11 @@
       <c r="N3" s="1">
         <v>2.0</v>
       </c>
-      <c r="O3" s="1" t="s">
-        <v>33</v>
+      <c r="O3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -1573,10 +1594,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>10</v>
@@ -1585,30 +1606,30 @@
         <v>9</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C2" s="1">
         <v>465.0</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E2" s="1">
         <v>5468.0</v>
@@ -1616,8 +1637,8 @@
       <c r="F2" s="1">
         <v>65465.0</v>
       </c>
-      <c r="G2" s="5" t="s">
-        <v>42</v>
+      <c r="G2" s="6" t="s">
+        <v>45</v>
       </c>
       <c r="H2" s="1">
         <v>55.0</v>

</xml_diff>

<commit_message>
FIX on deploy app; FIX on test; FIX on file column types
</commit_message>
<xml_diff>
--- a/test/fixtures/business_example_v2.xlsx
+++ b/test/fixtures/business_example_v2.xlsx
@@ -10,14 +10,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion1">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataSignature="AMtx7mjkLeq5sDy30Z7Dy9UQPiEyKs2yjA=="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataSignature="AMtx7mjMz9qQ/JfgxuYxYDChVlXYK7+5Qg=="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="50">
   <si>
     <t>businessName</t>
   </si>
@@ -97,6 +97,12 @@
     <t>sd541</t>
   </si>
   <si>
+    <t>Afghanistan</t>
+  </si>
+  <si>
+    <t>Badghis</t>
+  </si>
+  <si>
     <t>USD</t>
   </si>
   <si>
@@ -130,6 +136,9 @@
     <t>4q9wf8q9</t>
   </si>
   <si>
+    <t>name</t>
+  </si>
+  <si>
     <t>type</t>
   </si>
   <si>
@@ -146,6 +155,9 @@
   </si>
   <si>
     <t>workinghours</t>
+  </si>
+  <si>
+    <t>site 484</t>
   </si>
   <si>
     <t>some</t>
@@ -200,13 +212,13 @@
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left"/>
     </xf>
@@ -485,7 +497,7 @@
       <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
       <c r="P1" s="1" t="s">
@@ -505,7 +517,7 @@
       <c r="D2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F2" s="1" t="s">
@@ -526,40 +538,40 @@
       <c r="K2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="L2" s="4">
+      <c r="L2" s="3">
         <v>43862.0</v>
       </c>
-      <c r="M2" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="N2" s="1">
-        <v>2.0</v>
-      </c>
-      <c r="O2" s="2" t="s">
+      <c r="M2" s="4" t="s">
         <v>26</v>
       </c>
+      <c r="N2" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>28</v>
+      </c>
       <c r="P2" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>34</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>22</v>
@@ -568,7 +580,7 @@
         <v>1.223334444E9</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>24</v>
@@ -576,20 +588,20 @@
       <c r="K3" s="5">
         <v>5498.0</v>
       </c>
-      <c r="L3" s="4">
+      <c r="L3" s="3">
         <v>43862.0</v>
       </c>
-      <c r="M3" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="N3" s="1">
-        <v>2.0</v>
-      </c>
-      <c r="O3" s="2" t="s">
-        <v>35</v>
+      <c r="M3" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="N3" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -1587,60 +1599,66 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="6" width="8.71"/>
-    <col customWidth="1" min="7" max="7" width="23.0"/>
-    <col customWidth="1" min="8" max="26" width="8.71"/>
+    <col customWidth="1" min="1" max="7" width="8.71"/>
+    <col customWidth="1" min="8" max="8" width="23.0"/>
+    <col customWidth="1" min="9" max="27" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>39</v>
-      </c>
       <c r="F1" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="1">
+      <c r="D2" s="1">
         <v>465.0</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="E2" s="1">
+      <c r="E2" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F2" s="1">
         <v>5468.0</v>
       </c>
-      <c r="F2" s="1">
+      <c r="G2" s="1">
         <v>65465.0</v>
       </c>
-      <c r="G2" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="H2" s="1">
+      <c r="H2" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="I2" s="1">
         <v>55.0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
FIX on file import
</commit_message>
<xml_diff>
--- a/test/fixtures/business_example_v2.xlsx
+++ b/test/fixtures/business_example_v2.xlsx
@@ -1,14 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26006"/>
   <workbookPr/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6D940BF2-8E65-42CE-A3C7-6C197CBD3630}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Hoja1" sheetId="1" r:id="rId4"/>
-    <sheet state="visible" name="Hoja2" sheetId="2" r:id="rId5"/>
+    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="191028"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext uri="GoogleSheetsCustomDataVersion1">
       <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataSignature="AMtx7mjMz9qQ/JfgxuYxYDChVlXYK7+5Qg=="/>
     </ext>
@@ -17,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="53">
   <si>
     <t>businessName</t>
   </si>
@@ -67,6 +82,9 @@
     <t>password</t>
   </si>
   <si>
+    <t>address_1</t>
+  </si>
+  <si>
     <t>main</t>
   </si>
   <si>
@@ -109,6 +127,9 @@
     <t>89651sasf</t>
   </si>
   <si>
+    <t>address f</t>
+  </si>
+  <si>
     <t>gobal services inc</t>
   </si>
   <si>
@@ -134,6 +155,9 @@
   </si>
   <si>
     <t>4q9wf8q9</t>
+  </si>
+  <si>
+    <t>address j</t>
   </si>
   <si>
     <t>name</t>
@@ -172,23 +196,19 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="D/M/YYYY"/>
+    <numFmt numFmtId="164" formatCode="d/m/yyyy"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="2">
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <color theme="1"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
     </font>
@@ -198,49 +218,50 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -430,31 +451,31 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:Q1000"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="3" width="8.71"/>
-    <col customWidth="1" min="4" max="4" width="14.14"/>
-    <col customWidth="1" min="5" max="5" width="13.86"/>
-    <col customWidth="1" min="6" max="6" width="14.14"/>
-    <col customWidth="1" min="7" max="7" width="11.86"/>
-    <col customWidth="1" min="8" max="8" width="15.71"/>
-    <col customWidth="1" min="9" max="9" width="20.43"/>
-    <col customWidth="1" min="10" max="10" width="8.71"/>
-    <col customWidth="1" min="11" max="11" width="11.14"/>
-    <col customWidth="1" min="12" max="12" width="18.29"/>
-    <col customWidth="1" min="13" max="13" width="13.43"/>
-    <col customWidth="1" min="14" max="22" width="8.71"/>
+    <col min="1" max="3" width="8.7109375" customWidth="1"/>
+    <col min="4" max="4" width="14.140625" customWidth="1"/>
+    <col min="5" max="5" width="13.85546875" customWidth="1"/>
+    <col min="6" max="6" width="14.140625" customWidth="1"/>
+    <col min="7" max="7" width="11.85546875" customWidth="1"/>
+    <col min="8" max="8" width="15.7109375" customWidth="1"/>
+    <col min="9" max="9" width="20.42578125" customWidth="1"/>
+    <col min="10" max="10" width="8.7109375" customWidth="1"/>
+    <col min="11" max="11" width="11.140625" customWidth="1"/>
+    <col min="12" max="12" width="18.28515625" customWidth="1"/>
+    <col min="13" max="13" width="13.42578125" customWidth="1"/>
+    <col min="14" max="22" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:17">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -503,105 +524,114 @@
       <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="Q1" t="s">
+        <v>16</v>
+      </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:17">
       <c r="A2" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H2" s="1">
-        <v>1.223334444E9</v>
+        <v>1223334444</v>
       </c>
       <c r="I2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="L2" s="3">
+        <v>43862</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17">
+      <c r="A3" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="J2" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="K2" s="1" t="s">
+      <c r="H3" s="1">
+        <v>1223334444</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="J3" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="L2" s="3">
-        <v>43862.0</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="N2" s="4" t="s">
+      <c r="K3" s="4">
+        <v>5498</v>
+      </c>
+      <c r="L3" s="3">
+        <v>43862</v>
+      </c>
+      <c r="M3" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="O2" s="1" t="s">
+      <c r="N3" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="P2" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="H3" s="1">
-        <v>1.223334444E9</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="K3" s="5">
-        <v>5498.0</v>
-      </c>
-      <c r="L3" s="3">
-        <v>43862.0</v>
-      </c>
-      <c r="M3" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="N3" s="4" t="s">
-        <v>27</v>
-      </c>
       <c r="O3" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -1585,34 +1615,30 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
-  <printOptions/>
-  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:I1000"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="7" width="8.71"/>
-    <col customWidth="1" min="8" max="8" width="23.0"/>
-    <col customWidth="1" min="9" max="27" width="8.71"/>
+    <col min="1" max="7" width="8.7109375" customWidth="1"/>
+    <col min="8" max="8" width="23" customWidth="1"/>
+    <col min="9" max="27" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>10</v>
@@ -1621,45 +1647,45 @@
         <v>9</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:9">
       <c r="A2" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D2" s="1">
-        <v>465.0</v>
+        <v>465</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="F2" s="1">
-        <v>5468.0</v>
+        <v>5468</v>
       </c>
       <c r="G2" s="1">
-        <v>65465.0</v>
-      </c>
-      <c r="H2" s="6" t="s">
-        <v>49</v>
+        <v>65465</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>52</v>
       </c>
       <c r="I2" s="1">
-        <v>55.0</v>
+        <v>55</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -2643,9 +2669,7 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
-  <printOptions/>
-  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>